<commit_message>
Add new scripts for generating sticker orders and personal wraps
- Introduced `make_order.py` to automate the creation of sticker sheets and personal wraps for orders.
- Added `sticker_wrap.py` to generate custom wraps for each order, including customer details and design previews.
- Created `sticker_wrap_README.md` for documentation on usage and folder structure.
- Included necessary assets for branding and design in the project directory.
- Updated related documentation to reflect new processes and file structures.
</commit_message>
<xml_diff>
--- a/stikerts/projrct/updates/TestTrackingSheet.xlsx
+++ b/stikerts/projrct/updates/TestTrackingSheet.xlsx
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="206">
   <si>
     <t xml:space="preserve">Bin Sticker — Test Tracking Workbook</t>
   </si>
@@ -104,10 +104,10 @@
     <t xml:space="preserve">Free pre-purchase check for the kiss-cut machine upgrade path — confirms whether the DXF file imports cleanly into Silhouette Studio Basic (free) before you spend money on either the Portrait 4 or Joy Xtra. (CLOSED Sep 2026 — the Cricut Explore 5 was bought, so this comparison is moot.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Status (Sep 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test 6: the A6/C6 board-backed envelope is now row 5 (confirmed choice, still to be measured and transit-tested); the backing card and box are comparators. Corner Punch &amp; Peel-Nick: ON HOLD — bin sticker cutting is now Cricut cut-only for all sizes; the 3 Aug results are kept. Addendum 4: CLOSED. The Cricut Design Space SVG import check now sits in Addendum 6 of Bin-Sticker-Material-Test-Plan.md (no tab here yet).</t>
+    <t xml:space="preserve">Status (Oct 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test 6 complete: the A6/C6 board-backed envelope (single packs, Letter) and the AKAR A6/C6 box (2-4 packs, Large Letter) passed the Post Office counter check, drop/flex and post-to-self (2-day delivery). Weights and box measurements are on the 'Packing Results Oct 2026' tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Packing measurements - Oct 2026 (envelope + AKAR box)</t>
@@ -233,6 +233,9 @@
     <t xml:space="preserve">Note: 1 pack uses the envelope as a Letter (cheapest). Box rows assume loose packs (no envelopes); packs in envelopes add ~14g each and cross 100g sooner.</t>
   </si>
   <si>
+    <t xml:space="preserve">Note (Oct 2026): all weights on this tab were taken WITHOUT the personal paper wrap (~4.1g and ~0.5-0.6mm a pack). 4 wrapped packs would be about 98-100g, so the box cap is 3 wrapped packs until weighed. The 4-pack postage row assumes unwrapped packs.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Test 6 — Transit / Shipping Stress</t>
   </si>
   <si>
@@ -296,10 +299,16 @@
     <t xml:space="preserve">5. A6/C6 board-backed "Do Not Bend" envelope (confirmed choice)</t>
   </si>
   <si>
+    <t xml:space="preserve">&lt;5 (passed PO gauge)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y</t>
+  </si>
+  <si>
     <t xml:space="preserve">31g (envelope + 1 pack + tape)</t>
   </si>
   <si>
-    <t xml:space="preserve">letter (provisional) - packed thickness reported as under 4mm, not measured exactly; confirm at Post Office gauge</t>
+    <t xml:space="preserve">letter - passed Post Office counter check; posted Oct 2026. Exact mm not measured (reported under 4mm). Price charged not logged</t>
   </si>
   <si>
     <t xml:space="preserve">6. AKAR white A6/C6 Large Letter box (2-4 packs)</t>
@@ -308,7 +317,7 @@
     <t xml:space="preserve">57g (2 packs, taped); 82g (4 packs, tape not yet included)</t>
   </si>
   <si>
-    <t xml:space="preserve">large letter - 23mm leaves 2mm under the 25mm limit; cap at 4 packs</t>
+    <t xml:space="preserve">large letter - 23mm (2mm under the 25mm limit). Weights are WITHOUT the personal wrap: 4 packs 82g. The wrap adds ~4g a pack, so 4 wrapped packs would be ~98-100g - cap at 3 wrapped packs until 4 wrapped are weighed</t>
   </si>
   <si>
     <t xml:space="preserve">Drop / flex test (do first)</t>
@@ -326,7 +335,10 @@
     <t xml:space="preserve">Flex x5 (30°, 2s)</t>
   </si>
   <si>
-    <t xml:space="preserve">Oct 2026: tester reports packaging tested and good to go (no per-drop detail logged)</t>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 2026: all drops and flex passed (per tester)</t>
   </si>
   <si>
     <t xml:space="preserve">Post-to-self test</t>
@@ -347,7 +359,16 @@
     <t xml:space="preserve">Shift inside?</t>
   </si>
   <si>
-    <t xml:space="preserve">PENDING - to be posted via Click &amp; Drop (label printed in branch); log arrival results</t>
+    <t xml:space="preserve">Oct 2026 (date not logged)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 days after posting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass (none)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passed - arrived in 2 days via Click &amp; Drop, no creasing, corner damage or shifting (per tester)</t>
   </si>
   <si>
     <t xml:space="preserve">Decision</t>
@@ -356,7 +377,7 @@
     <t xml:space="preserve">Chosen packaging:</t>
   </si>
   <si>
-    <t xml:space="preserve">A6/C6 board-backed 'Do Not Bend' envelope for single packs (Letter, provisional); AKAR box for 2-4 packs (Large Letter) - pending Post Office gauge + post-to-self</t>
+    <t xml:space="preserve">CONFIRMED Oct 2026: A6/C6 board-backed 'Do Not Bend' envelope for single packs (Letter); AKAR box for 2-4 packs (Large Letter). Passed counter check, drop/flex and post-to-self.</t>
   </si>
   <si>
     <t xml:space="preserve">If backing card performs close to padded mailer/box → standout (Letter-rate + real protection). If it creases like flat wrap → the extra postage for mailer/box is buying real protection.</t>
@@ -368,6 +389,9 @@
     <t xml:space="preserve">Update Oct 2026: tape adds ~2g (box + 2 packs 55g -&gt; 57g; envelope unchanged at 31g). Tape used: ~30cm per envelope, ~45cm per box. Box weights: 2 packs 55g, 3 packs 69g, 4 packs 82g (~13-14g per pack). Labels are printed at the Post Office via Click &amp; Drop, so they are excluded from thickness/weight.</t>
   </si>
   <si>
+    <t xml:space="preserve">Update Oct 2026: Test 6 complete - envelope and AKAR box passed the Post Office counter check, all drop/flex tests and post-to-self (arrived in 2 days). Not logged: exact envelope thickness (mm), price charged at the counter, posting date.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Corner Punch &amp; Peel-Nick Check</t>
   </si>
   <si>
@@ -401,13 +425,7 @@
     <t xml:space="preserve">4mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass</t>
-  </si>
-  <si>
     <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y</t>
   </si>
   <si>
     <t xml:space="preserve">7mm</t>
@@ -887,7 +905,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -937,6 +955,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1353,7 +1375,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="58"/>
@@ -1825,6 +1847,11 @@
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
       <c r="E39" s="8"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13" t="s">
+        <v>57</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1845,7 +1872,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -1858,7 +1885,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1869,145 +1896,146 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" s="13" t="n">
+        <v>59</v>
+      </c>
+      <c r="B3" s="14" t="n">
         <v>46237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>59</v>
+      <c r="A5" s="15" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="B6" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="C6" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="D6" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="E6" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16" t="s">
+      <c r="F6" s="16" t="s">
         <v>66</v>
       </c>
+      <c r="G6" s="16"/>
+      <c r="H6" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="18" t="s">
+      <c r="A7" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="17" t="str">
+      <c r="B7" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="18" t="str">
         <f aca="false">IF(B7="","",IF(B7&lt;5,"Y","N"))</f>
         <v>N</v>
       </c>
-      <c r="D7" s="18"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="18" t="n">
+      <c r="A8" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="17" t="str">
+      <c r="C8" s="18" t="str">
         <f aca="false">IF(B8="","",IF(B8&lt;5,"Y","N"))</f>
         <v>Y</v>
       </c>
-      <c r="D8" s="18"/>
-      <c r="E8" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="F8" s="17" t="n">
+      <c r="D8" s="19"/>
+      <c r="E8" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="18" t="n">
         <v>0.91</v>
       </c>
-      <c r="G8" s="17" t="s">
-        <v>71</v>
+      <c r="G8" s="18" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="17" t="str">
+      <c r="A9" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="18" t="str">
         <f aca="false">IF(B9="","",IF(B9&lt;5,"Y","N"))</f>
         <v>N</v>
       </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" s="18" t="n">
+      <c r="A10" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="17" t="str">
+      <c r="C10" s="18" t="str">
         <f aca="false">IF(B10="","",IF(B10&lt;5,"Y","N"))</f>
         <v>Y</v>
       </c>
-      <c r="D10" s="18"/>
-      <c r="E10" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="F10" s="17" t="n">
+      <c r="D10" s="19"/>
+      <c r="E10" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="18" t="n">
         <v>1.55</v>
       </c>
-      <c r="G10" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="H10" s="19" t="s">
+      <c r="G10" s="18" t="s">
         <v>76</v>
       </c>
+      <c r="H10" s="20" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="17" t="str">
-        <f aca="false">IF(B11="","",IF(B11&lt;5,"Y","N"))</f>
-        <v/>
-      </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="17" t="s">
+      <c r="A11" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="B11" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="19"/>
+      <c r="E11" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="18" t="n">
         <v>0.91</v>
       </c>
-      <c r="G11" s="17" t="s">
-        <v>79</v>
+      <c r="G11" s="18" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12" s="20" t="n">
+        <v>83</v>
+      </c>
+      <c r="B12" s="21" t="n">
         <v>23</v>
       </c>
       <c r="C12" s="1" t="str">
@@ -2015,251 +2043,308 @@
         <v>N</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>1.55</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>83</v>
+      <c r="A13" s="15" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="E14" s="15" t="s">
+      <c r="A14" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15" t="s">
-        <v>66</v>
+      <c r="C14" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="21"/>
+      <c r="A15" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="21"/>
+      <c r="A16" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="22"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="21"/>
+      <c r="A17" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="21"/>
+      <c r="A18" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="22"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="21" t="s">
-        <v>88</v>
+      <c r="A19" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" s="18"/>
+      <c r="G19" s="22" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
-        <v>89</v>
+      <c r="A21" s="15" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="B22" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="F22" s="15" t="s">
+      <c r="A22" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="15" t="s">
-        <v>66</v>
+      <c r="C22" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="F22" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="G22" s="16" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="21"/>
+      <c r="A23" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="21"/>
+      <c r="A24" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="22"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="21"/>
+      <c r="A25" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="21"/>
+      <c r="A26" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="22"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="21" t="s">
-        <v>95</v>
+      <c r="A27" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="G27" s="22" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>101</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
-        <v>96</v>
+      <c r="A29" s="15" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B30" s="18" t="s">
-        <v>98</v>
+        <v>104</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="B31" s="22"/>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="22"/>
+      <c r="A31" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
     </row>
     <row r="32" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
+      <c r="A32" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
     </row>
     <row r="33" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
+      <c r="A33" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+    </row>
+    <row r="34" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="B34" s="24"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A34:G34"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B15:E19" type="list">
@@ -2300,7 +2385,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2308,184 +2393,184 @@
       <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="24" t="s">
-        <v>103</v>
+      <c r="A2" s="25" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B3" s="13" t="n">
+        <v>112</v>
+      </c>
+      <c r="B3" s="14" t="n">
         <v>46237</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>106</v>
+        <v>113</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
-        <v>107</v>
+      <c r="A6" s="15" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>66</v>
+      <c r="A7" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" s="21"/>
+      <c r="A8" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="E9" s="21"/>
+      <c r="A9" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="E10" s="21"/>
+      <c r="A10" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="E10" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>117</v>
+        <v>124</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
-        <v>119</v>
+      <c r="A14" s="15" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="B15" s="15" t="s">
+      <c r="A15" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" s="18"/>
+      <c r="E16" s="22"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="C15" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="D16" s="17"/>
-      <c r="E16" s="21"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="21"/>
+      <c r="C17" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="D17" s="18"/>
+      <c r="E17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="n">
+      <c r="A18" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="18" t="s">
-        <v>115</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="D18" s="17"/>
-      <c r="E18" s="21"/>
+      <c r="B18" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="D18" s="18"/>
+      <c r="E18" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>124</v>
+        <v>129</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>96</v>
+      <c r="A22" s="15" t="s">
+        <v>103</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="22" t="s">
-        <v>126</v>
-      </c>
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
+      <c r="A23" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2529,7 +2614,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2539,229 +2624,229 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B3" s="18"/>
+        <v>112</v>
+      </c>
+      <c r="B3" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
-        <v>128</v>
-      </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="A4" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>133</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>66</v>
+      <c r="A6" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="21"/>
+      <c r="A7" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="21"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="22"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="21"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="21"/>
+      <c r="A10" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="21"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="22"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="21"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="22"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="B13" s="17" t="s">
+      <c r="A13" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C13" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="C13" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="21"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="22"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="21"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="21"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="22"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="22"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="C16" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="21"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="21"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="21"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="22"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
-        <v>145</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>146</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="21"/>
+      <c r="A19" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="21"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="22"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="21"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
+      <c r="A23" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
+      <c r="A25" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2806,7 +2891,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2815,205 +2900,205 @@
       <c r="F1" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
+      <c r="A3" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
+        <v>157</v>
+      </c>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
       <c r="D5" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
+        <v>158</v>
+      </c>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
+      <c r="A7" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>154</v>
+      <c r="A9" s="15" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="B10" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="F10" s="15" t="s">
-        <v>160</v>
+      <c r="A10" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>161</v>
-      </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="A11" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
-        <v>162</v>
-      </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="A12" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="A13" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
-        <v>164</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="A14" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
+      <c r="A15" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
-        <v>166</v>
-      </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="A16" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
+      <c r="A17" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>168</v>
+      <c r="A19" s="15" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="B20" s="15" t="s">
-        <v>170</v>
-      </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15" t="s">
-        <v>66</v>
+      <c r="A20" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="21"/>
+      <c r="A21" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="B21" s="19"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="22"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
-        <v>172</v>
-      </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="21"/>
+      <c r="A22" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
-        <v>173</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="21"/>
+      <c r="A23" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
-        <v>174</v>
-      </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="21"/>
+      <c r="A24" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
-        <v>96</v>
+      <c r="A26" s="15" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
-        <v>175</v>
-      </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
+      <c r="A27" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3058,7 +3143,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3067,159 +3152,159 @@
       <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="24" t="s">
-        <v>177</v>
+      <c r="A2" s="25" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
+      <c r="A3" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>179</v>
+      <c r="A5" s="15" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>182</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>66</v>
+      <c r="A6" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>185</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="21"/>
+      <c r="A7" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="21"/>
+      <c r="A8" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="22"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>189</v>
+      <c r="A10" s="15" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="s">
-        <v>190</v>
-      </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
+      <c r="A11" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>192</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>193</v>
-      </c>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15" t="s">
-        <v>66</v>
+      <c r="A13" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>198</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="17" t="s">
-        <v>195</v>
-      </c>
-      <c r="D14" s="18"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="21"/>
+      <c r="A14" s="29" t="s">
+        <v>200</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="D14" s="19"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
-        <v>196</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="17" t="s">
-        <v>195</v>
-      </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="21"/>
+      <c r="A15" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="D15" s="19"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="22"/>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
-        <v>197</v>
-      </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="17" t="s">
-        <v>195</v>
-      </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="21"/>
+      <c r="A16" s="29" t="s">
+        <v>203</v>
+      </c>
+      <c r="B16" s="19"/>
+      <c r="C16" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="D16" s="19"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>96</v>
+      <c r="A18" s="15" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22" t="s">
-        <v>198</v>
-      </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="A19" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
+        <v>205</v>
+      </c>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>